<commit_message>
test evaluation of accuracy
</commit_message>
<xml_diff>
--- a/0_SELECT_ZIVE_DATA_2023/AtsisiuntimasZiveDuomenu/Atsisiusti_visi_anotuoti_duomenys/visi_zive_irasai_annot-Darb.xlsx
+++ b/0_SELECT_ZIVE_DATA_2023/AtsisiuntimasZiveDuomenu/Atsisiusti_visi_anotuoti_duomenys/visi_zive_irasai_annot-Darb.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kesju\DI\2025_ZIVEO\PROJECT_TRAIN_UNET\0_SELECT_ZIVE_DATA_2023\AtsisiuntimasZiveDuomenu\Atsisiusti_visi_anotuoti_duomenys\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40A7147A-640B-4B96-B0A3-E04BB772A037}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA540EEE-3233-4B21-BCE6-16B36E143237}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8751" uniqueCount="3919">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8751" uniqueCount="3920">
   <si>
     <t>filename</t>
   </si>
@@ -11781,6 +11781,9 @@
   </si>
   <si>
     <t>Normalizuotas įrašo vardas</t>
+  </si>
+  <si>
+    <t>mra</t>
   </si>
 </sst>
 </file>
@@ -12356,7 +12359,7 @@
         <v>19</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>20</v>
+        <v>3919</v>
       </c>
       <c r="Z1" s="1" t="s">
         <v>21</v>

</xml_diff>